<commit_message>
refactor(assess): move impact levers and headcount to L3 grain, generate L4 activities via LLM
Tower leads now author and dial at the L3 capability level — the upload
template carries L1/L2/L3 + headcount only, and the offshore + AI sliders
attach directly to each L3 row. L4 activities become display-only context:
seeded from the canonical map and (re)generated post-upload by a new
LLM-backed endpoint with a canonical-map fallback. Bumps assess program to
V4 with a one-pass migration that groups legacy per-L4 rows into per-L3
rows (cost-weighted dials, summed headcount, preserved L4 names).

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/assess-tower-template.xlsx
+++ b/public/assess-tower-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,21 +407,18 @@
         <v>L3</v>
       </c>
       <c r="C1" t="str">
-        <v>L4</v>
+        <v>FTE_onshore</v>
       </c>
       <c r="D1" t="str">
-        <v>FTE_onshore</v>
+        <v>FTE_offshore</v>
       </c>
       <c r="E1" t="str">
-        <v>FTE_offshore</v>
+        <v>contractor_onshore</v>
       </c>
       <c r="F1" t="str">
-        <v>contractor_onshore</v>
+        <v>contractor_offshore</v>
       </c>
       <c r="G1" t="str">
-        <v>contractor_offshore</v>
-      </c>
-      <c r="H1" t="str">
         <v>annual_spend_usd</v>
       </c>
     </row>
@@ -432,11 +429,11 @@
       <c r="B2" t="str">
         <v>Sub1</v>
       </c>
-      <c r="C2" t="str">
-        <v>Activity example 1</v>
+      <c r="C2">
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -444,10 +441,7 @@
       <c r="F2">
         <v>0</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="str">
+      <c r="G2" t="str">
         <v/>
       </c>
     </row>
@@ -456,30 +450,27 @@
         <v>PillarA</v>
       </c>
       <c r="B3" t="str">
-        <v>Sub1</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Activity example 2</v>
+        <v>Sub2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
       </c>
       <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>1</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3" t="str">
+      <c r="G3" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>